<commit_message>
CD-250: Update EDP schema
- Rename column `term_manifest_behavior`  to `term_access`

- Added new fields for the `version_tissue` manifest - `tissue type`, `weight`, `preservative`, `method_of_ preservation` and `time_to_preserve`

- Added `Project:ProjectId` `sapio_name` to the `study_id` field

- Revised regexes, error messages and reverted to title-case labels and  dropdown menu values to upper case.

- In the `edp_schema_template_v0.1.xlsx`,  instructions and the health and safety text were reworded
</commit_message>
<xml_diff>
--- a/edp/edp_schema_template_v0.1.xlsx
+++ b/edp/edp_schema_template_v0.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/edp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1949B029-BEAC-F54C-802B-550A6BC9C36C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A24CC8F3-532C-DC48-9517-9180F36FD079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18060" xr2:uid="{964001A8-9378-804A-8584-54773ECBCFFA}"/>
+    <workbookView xWindow="4980" yWindow="4240" windowWidth="30240" windowHeight="12520" activeTab="1" xr2:uid="{964001A8-9378-804A-8584-54773ECBCFFA}"/>
   </bookViews>
   <sheets>
     <sheet name="How to complete the manifest" sheetId="3" r:id="rId1"/>
@@ -139,10 +139,25 @@
     <t>Fields in blue are optional</t>
   </si>
   <si>
-    <t>Email address(es) of person(s) who final data should be sent to</t>
+    <t>Do you require samples to be returned to you (at your cost) on completion of the project?</t>
   </si>
   <si>
-    <t>Do you require samples to be returned to you (at your cost) on completion of the project?</t>
+    <t>SAMPLE DETAILS</t>
+  </si>
+  <si>
+    <t>For the use of Earlham Institute only - DO NOT EDIT</t>
+  </si>
+  <si>
+    <t>Do not edit the fields highlighted in grey because they are reserved for use by the Earlham Institute.</t>
+  </si>
+  <si>
+    <t>Instructions for completing the manifest</t>
+  </si>
+  <si>
+    <t>projects@earlham.ac.uk</t>
+  </si>
+  <si>
+    <t>Please complete this manifest and return it to the Project Management (PM) team by email before submitting your samples.</t>
   </si>
   <si>
     <r>
@@ -163,11 +178,11 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">
-By submitting this manifest to EI you are confirming that, if relevant, you have informed us of any potential health and safety risks associated with the samples. Please select </t>
+By submitting this manifest to the Earlham Insititue (EI), you are confirming that if relevant, you have informed us of any potential health and safety risks associated with the samples. Please select </t>
     </r>
     <r>
       <rPr>
-        <u/>
+        <b/>
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
@@ -184,9 +199,6 @@
       </rPr>
       <t xml:space="preserve"> (in the box to the right) to confirm you have read and understood this message.</t>
     </r>
-  </si>
-  <si>
-    <t>Please complete this manifest and return it to our Project Management team by email before submitting your samples.</t>
   </si>
   <si>
     <r>
@@ -207,7 +219,7 @@
     </r>
     <r>
       <rPr>
-        <u/>
+        <b/>
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
@@ -222,17 +234,17 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> column, in the </t>
+      <t xml:space="preserve"> column in the </t>
     </r>
     <r>
       <rPr>
-        <u/>
+        <b/>
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>Sample Details</t>
+      <t>SAMPLE DETAILS</t>
     </r>
     <r>
       <rPr>
@@ -241,36 +253,56 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> table of this manifest, for all samples submitted to EI.
+      <t xml:space="preserve"> section of this manifest for all samples submitted to EI.
+If you are unsure whether any of the regulations apply, please contact </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>projects@earlham.ac.uk</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.
  ♦ CITES - https://cites.org/eng
  ♦ Plant Health Regulations - https://www.gov.uk/guidance/plant-health-controls
  ♦ Human Tissue Act - https://www.hta.gov.uk/guidance-professionals/hta-legislation
  ♦ Nagoya Protocol - https://www.cbd.int/abs/about/ 
  ♦ UK GDPR &amp; The Data Protection Act 2018 - https://www.gov.uk/data-protection EU-GDPR https://gdpr.eu/tag/gdpr/ 
-     International data protection laws/regulations - https://www.dlapiperdataprotection.com/</t>
+    International data protection laws/regulations - https://www.dlapiperdataprotection.com/</t>
     </r>
   </si>
   <si>
-    <t>mailto:projects@earlham.ac.uk</t>
-  </si>
-  <si>
-    <t>SAMPLE DETAILS</t>
-  </si>
-  <si>
-    <t>For the use of Earlham Institute only - DO NOT EDIT</t>
-  </si>
-  <si>
-    <t>Do not edit fields highlighted in grey, these are for Earlham Institute use only</t>
-  </si>
-  <si>
-    <t>Instructions for completing the manifest.</t>
+    <r>
+      <t xml:space="preserve">Email address(es) of person(s) whom the sequencing data should be sent to
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Separate multiple addresses with a semicolon and a space</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -340,13 +372,6 @@
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FF0A0101"/>
       <name val="Arial"/>
@@ -355,12 +380,6 @@
     <font>
       <sz val="12"/>
       <color rgb="FFCC0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -384,7 +403,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -417,12 +436,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -439,6 +452,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="16">
     <border>
@@ -622,7 +647,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -635,16 +660,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -658,16 +683,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -689,10 +714,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -707,7 +732,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -765,14 +790,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -804,9 +829,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -826,13 +848,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -840,6 +873,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFC6E0B4"/>
+      <color rgb="FFBDD7EF"/>
+      <color rgb="FFDBF2D1"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1177,7 +1217,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" ht="21" x14ac:dyDescent="0.2">
       <c r="A1" s="19" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B1" s="20"/>
     </row>
@@ -1185,9 +1225,9 @@
       <c r="A2" s="21"/>
       <c r="B2" s="22"/>
     </row>
-    <row r="3" spans="1:2" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="23" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B3" s="24"/>
     </row>
@@ -1205,13 +1245,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="26" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="68"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="67"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -1247,11 +1287,11 @@
       <c r="R2" s="1"/>
     </row>
     <row r="3" spans="1:18" ht="21" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="71"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="70"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1269,12 +1309,12 @@
       <c r="R3" s="1"/>
     </row>
     <row r="4" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="75"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="74"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1285,20 +1325,20 @@
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
-      <c r="O4" s="76" t="s">
+      <c r="O4" s="79" t="s">
         <v>3</v>
       </c>
-      <c r="P4" s="73"/>
-      <c r="Q4" s="71"/>
+      <c r="P4" s="80"/>
+      <c r="Q4" s="81"/>
       <c r="R4" s="1"/>
     </row>
     <row r="5" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="72" t="s">
+      <c r="A5" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="77"/>
+      <c r="B5" s="72"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="75"/>
       <c r="E5" s="6" t="s">
         <v>5</v>
       </c>
@@ -1311,16 +1351,16 @@
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
-      <c r="O5" s="78" t="s">
+      <c r="O5" s="76" t="s">
         <v>6</v>
       </c>
-      <c r="P5" s="79"/>
-      <c r="Q5" s="80"/>
+      <c r="P5" s="77"/>
+      <c r="Q5" s="78"/>
       <c r="R5" s="1"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="30" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B6" s="31"/>
       <c r="C6" s="31"/>
@@ -1340,7 +1380,7 @@
       <c r="Q6" s="2"/>
       <c r="R6" s="1"/>
     </row>
-    <row r="7" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="23" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="32"/>
       <c r="B7" s="33"/>
       <c r="C7" s="33"/>
@@ -1362,7 +1402,7 @@
     </row>
     <row r="8" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="42"/>
       <c r="C8" s="42"/>
@@ -1384,7 +1424,7 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="43" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B9" s="44"/>
       <c r="C9" s="44"/>
@@ -1440,15 +1480,15 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="55" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P11" s="44"/>
       <c r="Q11" s="44"/>
       <c r="R11" s="45"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="56" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B12" s="57"/>
       <c r="C12" s="57"/>
@@ -1503,12 +1543,12 @@
       <c r="L14" s="11"/>
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
-      <c r="O14" s="65" t="s">
+      <c r="O14" s="82" t="s">
         <v>12</v>
       </c>
-      <c r="P14" s="39"/>
-      <c r="Q14" s="39"/>
-      <c r="R14" s="40"/>
+      <c r="P14" s="83"/>
+      <c r="Q14" s="83"/>
+      <c r="R14" s="84"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="59"/>
@@ -1670,7 +1710,7 @@
       <c r="Q22" s="13"/>
       <c r="R22" s="1"/>
     </row>
-    <row r="23" spans="1:18" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="62"/>
       <c r="B23" s="63"/>
       <c r="C23" s="63"/>
@@ -1732,7 +1772,7 @@
     </row>
     <row r="26" spans="1:18" ht="20" x14ac:dyDescent="0.2">
       <c r="A26" s="25" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="27"/>
@@ -1754,7 +1794,7 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" s="28" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B27" s="29"/>
       <c r="C27" s="29"/>
@@ -1795,7 +1835,7 @@
     <mergeCell ref="A9:K11"/>
     <mergeCell ref="L9:L11"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please select" sqref="L8" xr:uid="{5295E0F2-B1D8-1D4A-9C6B-C01C8ABCA05C}">
       <formula1>"YES,NO"</formula1>
     </dataValidation>
@@ -1808,9 +1848,10 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="O14:Q14" r:id="rId1" display="mailto:projects@earlham.ac.uk" xr:uid="{49881876-F596-AF42-A642-110708396225}"/>
-    <hyperlink ref="O14" r:id="rId2" xr:uid="{7A0622C2-AB1B-5649-A342-F913056CB9F6}"/>
+    <hyperlink ref="O14" r:id="rId2" display="mailto:projects@earlham.ac.uk" xr:uid="{7A0622C2-AB1B-5649-A342-F913056CB9F6}"/>
+    <hyperlink ref="O14:R14" r:id="rId3" display="projects@earlham.ac.uk" xr:uid="{A88255CC-B8C3-A149-AD45-1D5DF6AEA7AC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId3"/>
+  <legacyDrawing r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>